<commit_message>
1. Reverted scenario name back to "H2 heavy" to avoid duplication of files and data. 2. Corrected fuel prices and emissions for "H2 heavy" scenario. 3. Updated DH demand data (copy from demanddata_DH_own_projection). 4. Polished summary sheet in H2 heavy.xlsx.
</commit_message>
<xml_diff>
--- a/src_files/data_files/emissiondata_maf2020.xlsx
+++ b/src_files/data_files/emissiondata_maf2020.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\backbone\north_european_model (2IMatch)\src_files\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{925790C0-EADE-48EE-8182-E38B41CD96D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4BF835-BDBB-464C-ABA4-0AAEAF7A0307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="17520" xr2:uid="{3E3DEAD5-6055-4DB8-B424-EEC0B5E366CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{3E3DEAD5-6055-4DB8-B424-EEC0B5E366CE}"/>
   </bookViews>
   <sheets>
     <sheet name="emissiondata" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="10">
   <si>
     <t>CO2</t>
   </si>
@@ -64,9 +64,6 @@
   </si>
   <si>
     <t>group</t>
-  </si>
-  <si>
-    <t>H2 balanced</t>
   </si>
   <si>
     <t>ETS-CO2</t>
@@ -503,7 +500,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2">
         <v>105</v>
@@ -520,7 +517,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E3">
         <v>140</v>
@@ -537,7 +534,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E4">
         <v>120</v>
@@ -554,28 +551,14 @@
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5">
-        <v>105</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>2035</v>
-      </c>
-      <c r="C6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>105</v>
-      </c>
+      <c r="A6" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>